<commit_message>
feat: upgrade Excel sheet building-level grouping logic and update all assets
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-Park College.xlsx
+++ b/files/九龙-九龙塘-Park College.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="销控汇总明细" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Park College 销控表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Park College" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,14 +44,19 @@
     </font>
     <font>
       <name val="Microsoft YaHei"/>
-      <color rgb="007F7F7F"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
       <b val="1"/>
-      <color rgb="007F7F7F"/>
-      <sz val="11"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
@@ -63,7 +68,7 @@
       <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="00004D00"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
@@ -74,7 +79,7 @@
       <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="00002060"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
@@ -85,7 +90,7 @@
       <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="00660000"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Microsoft YaHei"/>
@@ -95,9 +100,30 @@
     </font>
     <font>
       <name val="Microsoft YaHei"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
       <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
+      <color rgb="007F7F7F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00660000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00004D00"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="9">
@@ -145,8 +171,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E5E5E5"/>
-        <bgColor rgb="00E5E5E5"/>
+        <fgColor rgb="00E8E8E8"/>
+        <bgColor rgb="00E8E8E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -176,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -193,19 +219,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -223,13 +237,37 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -607,7 +645,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
@@ -1200,195 +1238,195 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Park College - Park College 销控网格图</t>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Park College 销控网格图</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>总套数</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>在售 (Sale)</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>已定价未售</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>已售 (Sold)</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>暂停销售</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>待售 (Pending)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>11 套</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>2 套</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>9 套</t>
-        </is>
-      </c>
-      <c r="E3" s="15" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>0 套</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>楼层\房号</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>楼层</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>GV</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="65" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>7&amp;8/F</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>7&amp;8</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>A | 3040呎 (4+房)
-$12,800万
+$12800万
 $42,105/呎
 (已售)</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>B | 3022呎 (4+房)
-$15,000万
+$15000万
 $49,636/呎
 (已售)</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr"/>
-    </row>
-    <row r="7" ht="65" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>6/F</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr"/>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>A | 1478呎 (3房)
-$6,000万
+$6000万
 $40,595/呎
 (已售)</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>B | 1463呎 (3房)
-$6,000万
+$6000万
 $41,012/呎
 (已售)</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr"/>
-    </row>
-    <row r="8" ht="65" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>5/F</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr"/>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>A | 1478呎 (3房)
-$5,900万
+$5900万
 $39,919/呎
 (已售)</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>B | 1463呎 (3房)
-$5,900万
+$5900万
 $40,328/呎
 (已售)</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr"/>
-    </row>
-    <row r="9" ht="65" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>3/F</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr"/>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>A | 1478呎 (3房)
-$6,000万
+$6000万
 $40,595/呎
 (已售)</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>B | 1463呎 (3房)
 招标单位
@@ -1396,41 +1434,41 @@
 (在售)</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr"/>
-    </row>
-    <row r="10" ht="65" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2/F</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr"/>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>A | 1405呎 (3房)
-$6,300万
+$6300万
 $44,840/呎
 (已售)</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>B | 1390呎 (3房)
-$6,000万
+$6000万
 $43,165/呎
 (已售)</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr"/>
-    </row>
-    <row r="11" ht="65" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>G&amp;1/F</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="inlineStr"/>
-      <c r="C11" s="17" t="inlineStr"/>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr"/>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>G&amp;1</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr"/>
+      <c r="C10" s="21" t="inlineStr"/>
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>GV | 3060呎 (4+房)
 招标单位
@@ -1441,7 +1479,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>